<commit_message>
fixed issues with education data
</commit_message>
<xml_diff>
--- a/Education/2024_Secondary_Schools_Population.xlsx
+++ b/Education/2024_Secondary_Schools_Population.xlsx
@@ -34,22 +34,22 @@
     <t>2023/2024</t>
   </si>
   <si>
-    <t>JSS 1</t>
+    <t>JSS I</t>
   </si>
   <si>
-    <t>JSS 2</t>
+    <t>JSS II</t>
   </si>
   <si>
-    <t>JSS 3</t>
+    <t>JSS III</t>
   </si>
   <si>
-    <t>SSS 1</t>
+    <t>SSS I</t>
   </si>
   <si>
-    <t>SSS 2</t>
+    <t>SSS II</t>
   </si>
   <si>
-    <t>SSS 3</t>
+    <t>SSS III</t>
   </si>
   <si>
     <t>Male</t>

</xml_diff>